<commit_message>
feat: completar listado de tenants M02
</commit_message>
<xml_diff>
--- a/docs/Cronograma_M_Panel_Maestro_MVS_Commerce.xlsx
+++ b/docs/Cronograma_M_Panel_Maestro_MVS_Commerce.xlsx
@@ -111,22 +111,22 @@
     <t>Listado global de tenants con búsqueda, estado, propietario, plan, sucursales usadas/límite, módulos y usuarios.</t>
   </si>
   <si>
+    <t>MVS puede supervisar miles de empresas desde una sola vista.</t>
+  </si>
+  <si>
+    <t>Buscar/filtrar empresa y ver sucursales usadas/límite, estado, propietario, plan, módulos y usuarios sin entrar al tenant. Evidencia: M02PlatformTenantListTest + PlatformAdminTest + M01SaaSLicensingTest.</t>
+  </si>
+  <si>
+    <t>M03</t>
+  </si>
+  <si>
+    <t>Alta comercial</t>
+  </si>
+  <si>
+    <t>Reemplazar el alta operativa de 7 pasos del Panel Maestro por alta mínima de tenant/licencia: nombre de referencia, propietario, plan, branch_limit, módulos y estado.</t>
+  </si>
+  <si>
     <t>PENDIENTE</t>
-  </si>
-  <si>
-    <t>MVS puede supervisar miles de empresas desde una sola vista.</t>
-  </si>
-  <si>
-    <t>Buscar/filtrar empresa y ver 2/2 sucursales, estado, propietario y módulos sin entrar al tenant.</t>
-  </si>
-  <si>
-    <t>M03</t>
-  </si>
-  <si>
-    <t>Alta comercial</t>
-  </si>
-  <si>
-    <t>Reemplazar el alta operativa de 7 pasos del Panel Maestro por alta mínima de tenant/licencia: nombre de referencia, propietario, plan, branch_limit, módulos y estado.</t>
   </si>
   <si>
     <t>MVS crea el contrato/acceso, no llena datos fiscales ni operación del cliente.</t>
@@ -942,33 +942,33 @@
         <v>17</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="F10" s="8" t="s">
         <v>22</v>
       </c>
       <c r="G10" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="H10" s="8" t="s">
         <v>32</v>
-      </c>
-      <c r="H10" s="8" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="11" spans="1:8">
       <c r="A11" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="B11" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="C11" s="8" t="s">
         <v>35</v>
-      </c>
-      <c r="C11" s="8" t="s">
-        <v>36</v>
       </c>
       <c r="D11" s="8" t="s">
         <v>17</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="F11" s="8" t="s">
         <v>22</v>
@@ -994,10 +994,10 @@
         <v>17</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G12" s="8" t="s">
         <v>42</v>
@@ -1020,7 +1020,7 @@
         <v>17</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="F13" s="8" t="s">
         <v>39</v>
@@ -1046,7 +1046,7 @@
         <v>17</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="F14" s="8" t="s">
         <v>52</v>
@@ -1072,7 +1072,7 @@
         <v>17</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="F15" s="8" t="s">
         <v>22</v>
@@ -1098,7 +1098,7 @@
         <v>63</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="F16" s="8" t="s">
         <v>28</v>
@@ -1124,7 +1124,7 @@
         <v>63</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="F17" s="8" t="s">
         <v>69</v>
@@ -1150,7 +1150,7 @@
         <v>17</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="F18" s="8" t="s">
         <v>75</v>
@@ -1176,7 +1176,7 @@
         <v>63</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="F19" s="8" t="s">
         <v>81</v>
@@ -1202,7 +1202,7 @@
         <v>17</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="F20" s="8" t="s">
         <v>87</v>

</xml_diff>

<commit_message>
feat: completar alta comercial M03
</commit_message>
<xml_diff>
--- a/docs/Cronograma_M_Panel_Maestro_MVS_Commerce.xlsx
+++ b/docs/Cronograma_M_Panel_Maestro_MVS_Commerce.xlsx
@@ -126,22 +126,22 @@
     <t>Reemplazar el alta operativa de 7 pasos del Panel Maestro por alta mínima de tenant/licencia: nombre de referencia, propietario, plan, branch_limit, módulos y estado.</t>
   </si>
   <si>
+    <t>MVS crea el contrato/acceso, no llena datos fiscales ni operación del cliente.</t>
+  </si>
+  <si>
+    <t>Crea tenant sin cédula, dirección, sucursales ni cajas; propietario inactivo y contrato listos para activación/onboarding. Evidencia: M03CommercialTenantOnboardingTest + M01SaaSLicensingTest + PlatformAdminTest (19 pruebas, 113 aserciones).</t>
+  </si>
+  <si>
+    <t>M04</t>
+  </si>
+  <si>
+    <t>Acceso propietario</t>
+  </si>
+  <si>
+    <t>Crear invitación/activación segura para el propietario del tenant y primer ingreso obligatorio al onboarding.</t>
+  </si>
+  <si>
     <t>PENDIENTE</t>
-  </si>
-  <si>
-    <t>MVS crea el contrato/acceso, no llena datos fiscales ni operación del cliente.</t>
-  </si>
-  <si>
-    <t>Crear tenant sin cédula/direcciones/cajas; queda listo para que el propietario complete onboarding.</t>
-  </si>
-  <si>
-    <t>M04</t>
-  </si>
-  <si>
-    <t>Acceso propietario</t>
-  </si>
-  <si>
-    <t>Crear invitación/activación segura para el propietario del tenant y primer ingreso obligatorio al onboarding.</t>
   </si>
   <si>
     <t>El propietario recibe acceso propio y no puede entrar al Panel Maestro.</t>
@@ -968,33 +968,33 @@
         <v>17</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="F11" s="8" t="s">
         <v>22</v>
       </c>
       <c r="G11" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="H11" s="8" t="s">
         <v>37</v>
-      </c>
-      <c r="H11" s="8" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="12" spans="1:8">
       <c r="A12" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="B12" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="B12" s="8" t="s">
+      <c r="C12" s="8" t="s">
         <v>40</v>
-      </c>
-      <c r="C12" s="8" t="s">
-        <v>41</v>
       </c>
       <c r="D12" s="8" t="s">
         <v>17</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="F12" s="8" t="s">
         <v>33</v>
@@ -1020,10 +1020,10 @@
         <v>17</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G13" s="8" t="s">
         <v>47</v>
@@ -1046,7 +1046,7 @@
         <v>17</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="F14" s="8" t="s">
         <v>52</v>
@@ -1072,7 +1072,7 @@
         <v>17</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="F15" s="8" t="s">
         <v>22</v>
@@ -1098,7 +1098,7 @@
         <v>63</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="F16" s="8" t="s">
         <v>28</v>
@@ -1124,7 +1124,7 @@
         <v>63</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="F17" s="8" t="s">
         <v>69</v>
@@ -1150,7 +1150,7 @@
         <v>17</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="F18" s="8" t="s">
         <v>75</v>
@@ -1176,7 +1176,7 @@
         <v>63</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="F19" s="8" t="s">
         <v>81</v>
@@ -1202,7 +1202,7 @@
         <v>17</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="F20" s="8" t="s">
         <v>87</v>

</xml_diff>

<commit_message>
feat: completar activacion de propietario M04
</commit_message>
<xml_diff>
--- a/docs/Cronograma_M_Panel_Maestro_MVS_Commerce.xlsx
+++ b/docs/Cronograma_M_Panel_Maestro_MVS_Commerce.xlsx
@@ -141,22 +141,22 @@
     <t>Crear invitación/activación segura para el propietario del tenant y primer ingreso obligatorio al onboarding.</t>
   </si>
   <si>
+    <t>El propietario recibe acceso propio y no puede entrar al Panel Maestro.</t>
+  </si>
+  <si>
+    <t>Propietario recibe token personal, hash, expirable y single-use; activa cuenta tenant al definir clave y no accede al Panel Maestro. Evidencia: M04TenantOwnerInvitationTest + regresión M03/onboarding (9 pruebas, 62 aserciones).</t>
+  </si>
+  <si>
+    <t>M05</t>
+  </si>
+  <si>
+    <t>Onboarding tenant</t>
+  </si>
+  <si>
+    <t>Mover/reutilizar el flujo de empresa, identidad, primera sucursal y configuración para que lo complete el propietario del tenant.</t>
+  </si>
+  <si>
     <t>PENDIENTE</t>
-  </si>
-  <si>
-    <t>El propietario recibe acceso propio y no puede entrar al Panel Maestro.</t>
-  </si>
-  <si>
-    <t>Cuenta nueva entra al onboarding de su tenant; Platform Admin sigue separado.</t>
-  </si>
-  <si>
-    <t>M05</t>
-  </si>
-  <si>
-    <t>Onboarding tenant</t>
-  </si>
-  <si>
-    <t>Mover/reutilizar el flujo de empresa, identidad, primera sucursal y configuración para que lo complete el propietario del tenant.</t>
   </si>
   <si>
     <t>El cliente completa sus datos legales y operativos sin intervención de MVS.</t>
@@ -994,33 +994,33 @@
         <v>17</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>41</v>
+        <v>25</v>
       </c>
       <c r="F12" s="8" t="s">
         <v>33</v>
       </c>
       <c r="G12" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="H12" s="8" t="s">
         <v>42</v>
-      </c>
-      <c r="H12" s="8" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="13" spans="1:8">
       <c r="A13" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="B13" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="B13" s="8" t="s">
+      <c r="C13" s="8" t="s">
         <v>45</v>
-      </c>
-      <c r="C13" s="8" t="s">
-        <v>46</v>
       </c>
       <c r="D13" s="8" t="s">
         <v>17</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="F13" s="8" t="s">
         <v>38</v>
@@ -1046,7 +1046,7 @@
         <v>17</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="F14" s="8" t="s">
         <v>52</v>
@@ -1072,7 +1072,7 @@
         <v>17</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="F15" s="8" t="s">
         <v>22</v>
@@ -1098,7 +1098,7 @@
         <v>63</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="F16" s="8" t="s">
         <v>28</v>
@@ -1124,7 +1124,7 @@
         <v>63</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="F17" s="8" t="s">
         <v>69</v>
@@ -1150,7 +1150,7 @@
         <v>17</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="F18" s="8" t="s">
         <v>75</v>
@@ -1176,7 +1176,7 @@
         <v>63</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="F19" s="8" t="s">
         <v>81</v>
@@ -1202,7 +1202,7 @@
         <v>17</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="F20" s="8" t="s">
         <v>87</v>

</xml_diff>

<commit_message>
feat: completar onboarding tenant M05
</commit_message>
<xml_diff>
--- a/docs/Cronograma_M_Panel_Maestro_MVS_Commerce.xlsx
+++ b/docs/Cronograma_M_Panel_Maestro_MVS_Commerce.xlsx
@@ -156,22 +156,22 @@
     <t>Mover/reutilizar el flujo de empresa, identidad, primera sucursal y configuración para que lo complete el propietario del tenant.</t>
   </si>
   <si>
+    <t>El cliente completa sus datos legales y operativos sin intervención de MVS.</t>
+  </si>
+  <si>
+    <t>Primer ingreso exige completar el mismo tenant y primera sucursal antes del dashboard; conserva licencia/módulos. Evidencia: M05TenantOnboardingTest + regresión M04/onboarding/aprovisionamiento (14 pruebas, 78 aserciones).</t>
+  </si>
+  <si>
+    <t>M06</t>
+  </si>
+  <si>
+    <t>Sucursales</t>
+  </si>
+  <si>
+    <t>Aplicar branch_limit en creación de sucursales y permitir al Platform Admin aumentarlo/reducirlo.</t>
+  </si>
+  <si>
     <t>PENDIENTE</t>
-  </si>
-  <si>
-    <t>El cliente completa sus datos legales y operativos sin intervención de MVS.</t>
-  </si>
-  <si>
-    <t>Primer ingreso exige completar empresa + primera sucursal antes del dashboard.</t>
-  </si>
-  <si>
-    <t>M06</t>
-  </si>
-  <si>
-    <t>Sucursales</t>
-  </si>
-  <si>
-    <t>Aplicar branch_limit en creación de sucursales y permitir al Platform Admin aumentarlo/reducirlo.</t>
   </si>
   <si>
     <t>M01,M05</t>
@@ -1020,33 +1020,33 @@
         <v>17</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>46</v>
+        <v>25</v>
       </c>
       <c r="F13" s="8" t="s">
         <v>38</v>
       </c>
       <c r="G13" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="H13" s="8" t="s">
         <v>47</v>
-      </c>
-      <c r="H13" s="8" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="14" spans="1:8">
       <c r="A14" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="B14" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="B14" s="8" t="s">
+      <c r="C14" s="8" t="s">
         <v>50</v>
-      </c>
-      <c r="C14" s="8" t="s">
-        <v>51</v>
       </c>
       <c r="D14" s="8" t="s">
         <v>17</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="F14" s="8" t="s">
         <v>52</v>
@@ -1072,7 +1072,7 @@
         <v>17</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="F15" s="8" t="s">
         <v>22</v>
@@ -1098,7 +1098,7 @@
         <v>63</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="F16" s="8" t="s">
         <v>28</v>
@@ -1124,7 +1124,7 @@
         <v>63</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="F17" s="8" t="s">
         <v>69</v>
@@ -1150,7 +1150,7 @@
         <v>17</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="F18" s="8" t="s">
         <v>75</v>
@@ -1176,7 +1176,7 @@
         <v>63</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="F19" s="8" t="s">
         <v>81</v>
@@ -1202,7 +1202,7 @@
         <v>17</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="F20" s="8" t="s">
         <v>87</v>

</xml_diff>

<commit_message>
test: completar limite de sucursales M06
</commit_message>
<xml_diff>
--- a/docs/Cronograma_M_Panel_Maestro_MVS_Commerce.xlsx
+++ b/docs/Cronograma_M_Panel_Maestro_MVS_Commerce.xlsx
@@ -171,25 +171,25 @@
     <t>Aplicar branch_limit en creación de sucursales y permitir al Platform Admin aumentarlo/reducirlo.</t>
   </si>
   <si>
+    <t>M01,M05</t>
+  </si>
+  <si>
+    <t>El cliente crea sucursales hasta el límite contratado.</t>
+  </si>
+  <si>
+    <t>Límite 2 permite dos, bloquea tercera; al subir a 3 desde Panel Maestro vuelve a permitir. Reducir no borra sucursales. Evidencia: CustomerOnboardingAndBranchesTest + licencia/M01 (16 pruebas, 85 aserciones).</t>
+  </si>
+  <si>
+    <t>M07</t>
+  </si>
+  <si>
+    <t>Módulos</t>
+  </si>
+  <si>
+    <t>Aplicar módulos licenciados a navegación, rutas/permisos y capacidades; Platform Admin puede activar/desactivar módulos.</t>
+  </si>
+  <si>
     <t>PENDIENTE</t>
-  </si>
-  <si>
-    <t>M01,M05</t>
-  </si>
-  <si>
-    <t>El cliente crea sucursales hasta el límite contratado.</t>
-  </si>
-  <si>
-    <t>Con límite 2 permite dos; bloquea la tercera; al subir límite desde Panel Maestro vuelve a permitir.</t>
-  </si>
-  <si>
-    <t>M07</t>
-  </si>
-  <si>
-    <t>Módulos</t>
-  </si>
-  <si>
-    <t>Aplicar módulos licenciados a navegación, rutas/permisos y capacidades; Platform Admin puede activar/desactivar módulos.</t>
   </si>
   <si>
     <t>El tenant solo usa módulos contratados y no puede auto-habilitarlos.</t>
@@ -1046,33 +1046,33 @@
         <v>17</v>
       </c>
       <c r="E14" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="F14" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="F14" s="8" t="s">
+      <c r="G14" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="G14" s="8" t="s">
+      <c r="H14" s="8" t="s">
         <v>53</v>
-      </c>
-      <c r="H14" s="8" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="15" spans="1:8">
       <c r="A15" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="B15" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="B15" s="8" t="s">
+      <c r="C15" s="8" t="s">
         <v>56</v>
-      </c>
-      <c r="C15" s="8" t="s">
-        <v>57</v>
       </c>
       <c r="D15" s="8" t="s">
         <v>17</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="F15" s="8" t="s">
         <v>22</v>
@@ -1098,7 +1098,7 @@
         <v>63</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="F16" s="8" t="s">
         <v>28</v>
@@ -1124,7 +1124,7 @@
         <v>63</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="F17" s="8" t="s">
         <v>69</v>
@@ -1150,7 +1150,7 @@
         <v>17</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="F18" s="8" t="s">
         <v>75</v>
@@ -1176,7 +1176,7 @@
         <v>63</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="F19" s="8" t="s">
         <v>81</v>
@@ -1202,7 +1202,7 @@
         <v>17</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="F20" s="8" t="s">
         <v>87</v>

</xml_diff>

<commit_message>
test: completar modulos licenciados M07
</commit_message>
<xml_diff>
--- a/docs/Cronograma_M_Panel_Maestro_MVS_Commerce.xlsx
+++ b/docs/Cronograma_M_Panel_Maestro_MVS_Commerce.xlsx
@@ -189,25 +189,25 @@
     <t>Aplicar módulos licenciados a navegación, rutas/permisos y capacidades; Platform Admin puede activar/desactivar módulos.</t>
   </si>
   <si>
+    <t>El tenant solo usa módulos contratados y no puede auto-habilitarlos.</t>
+  </si>
+  <si>
+    <t>Módulo desactivado no aparece ni es accesible; al activarlo vuelve según permisos sin alterarlos. Tenant sin ruta de auto-habilitación. Evidencia: CompanyModuleAccessTest + M01/roles/navegación (27 pruebas, 105 aserciones).</t>
+  </si>
+  <si>
+    <t>M08</t>
+  </si>
+  <si>
+    <t>Ciclo de vida</t>
+  </si>
+  <si>
+    <t>Permitir activar, suspender, reactivar y cancelar tenant desde Panel Maestro con reglas seguras.</t>
+  </si>
+  <si>
+    <t>Alta</t>
+  </si>
+  <si>
     <t>PENDIENTE</t>
-  </si>
-  <si>
-    <t>El tenant solo usa módulos contratados y no puede auto-habilitarlos.</t>
-  </si>
-  <si>
-    <t>Módulo desactivado no aparece ni es accesible por URL; al activarlo queda disponible según permisos.</t>
-  </si>
-  <si>
-    <t>M08</t>
-  </si>
-  <si>
-    <t>Ciclo de vida</t>
-  </si>
-  <si>
-    <t>Permitir activar, suspender, reactivar y cancelar tenant desde Panel Maestro con reglas seguras.</t>
-  </si>
-  <si>
-    <t>Alta</t>
   </si>
   <si>
     <t>MVS controla el acceso comercial sin borrar datos del cliente.</t>
@@ -1072,33 +1072,33 @@
         <v>17</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>57</v>
+        <v>25</v>
       </c>
       <c r="F15" s="8" t="s">
         <v>22</v>
       </c>
       <c r="G15" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="H15" s="8" t="s">
         <v>58</v>
-      </c>
-      <c r="H15" s="8" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="16" spans="1:8">
       <c r="A16" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="B16" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="B16" s="8" t="s">
+      <c r="C16" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="C16" s="8" t="s">
+      <c r="D16" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="D16" s="8" t="s">
+      <c r="E16" s="8" t="s">
         <v>63</v>
-      </c>
-      <c r="E16" s="8" t="s">
-        <v>57</v>
       </c>
       <c r="F16" s="8" t="s">
         <v>28</v>
@@ -1121,10 +1121,10 @@
         <v>68</v>
       </c>
       <c r="D17" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="E17" s="8" t="s">
         <v>63</v>
-      </c>
-      <c r="E17" s="8" t="s">
-        <v>57</v>
       </c>
       <c r="F17" s="8" t="s">
         <v>69</v>
@@ -1150,7 +1150,7 @@
         <v>17</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="F18" s="8" t="s">
         <v>75</v>
@@ -1173,10 +1173,10 @@
         <v>80</v>
       </c>
       <c r="D19" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="E19" s="8" t="s">
         <v>63</v>
-      </c>
-      <c r="E19" s="8" t="s">
-        <v>57</v>
       </c>
       <c r="F19" s="8" t="s">
         <v>81</v>
@@ -1202,7 +1202,7 @@
         <v>17</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="F20" s="8" t="s">
         <v>87</v>

</xml_diff>

<commit_message>
test: validar ciclo de vida M08
</commit_message>
<xml_diff>
--- a/docs/Cronograma_M_Panel_Maestro_MVS_Commerce.xlsx
+++ b/docs/Cronograma_M_Panel_Maestro_MVS_Commerce.xlsx
@@ -207,22 +207,22 @@
     <t>Alta</t>
   </si>
   <si>
+    <t>MVS controla el acceso comercial sin borrar datos del cliente.</t>
+  </si>
+  <si>
+    <t>Suspendido/cancelado no opera; reactivación restaura acceso sin destruir empresa, sucursales ni datos. Evidencia: CompanyLicenseTest + M01 + PlatformAdminTest (21 pruebas, 116 aserciones).</t>
+  </si>
+  <si>
+    <t>M09</t>
+  </si>
+  <si>
+    <t>Detalle tenant</t>
+  </si>
+  <si>
+    <t>Crear ficha administrativa global: licencia, módulos, sucursales, usuarios, consumo de límites, fechas y acciones de administración.</t>
+  </si>
+  <si>
     <t>PENDIENTE</t>
-  </si>
-  <si>
-    <t>MVS controla el acceso comercial sin borrar datos del cliente.</t>
-  </si>
-  <si>
-    <t>Tenant suspendido no opera; reactivación restaura acceso; no se destruyen datos.</t>
-  </si>
-  <si>
-    <t>M09</t>
-  </si>
-  <si>
-    <t>Detalle tenant</t>
-  </si>
-  <si>
-    <t>Crear ficha administrativa global: licencia, módulos, sucursales, usuarios, consumo de límites, fechas y acciones de administración.</t>
   </si>
   <si>
     <t>M02,M06,M07,M08</t>
@@ -1098,33 +1098,33 @@
         <v>62</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>63</v>
+        <v>25</v>
       </c>
       <c r="F16" s="8" t="s">
         <v>28</v>
       </c>
       <c r="G16" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="H16" s="8" t="s">
         <v>64</v>
-      </c>
-      <c r="H16" s="8" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="17" spans="1:8">
       <c r="A17" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="B17" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="B17" s="8" t="s">
+      <c r="C17" s="8" t="s">
         <v>67</v>
-      </c>
-      <c r="C17" s="8" t="s">
-        <v>68</v>
       </c>
       <c r="D17" s="8" t="s">
         <v>62</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="F17" s="8" t="s">
         <v>69</v>
@@ -1150,7 +1150,7 @@
         <v>17</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="F18" s="8" t="s">
         <v>75</v>
@@ -1176,7 +1176,7 @@
         <v>62</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="F19" s="8" t="s">
         <v>81</v>
@@ -1202,7 +1202,7 @@
         <v>17</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="F20" s="8" t="s">
         <v>87</v>

</xml_diff>

<commit_message>
docs: completar ficha administrativa M09
</commit_message>
<xml_diff>
--- a/docs/Cronograma_M_Panel_Maestro_MVS_Commerce.xlsx
+++ b/docs/Cronograma_M_Panel_Maestro_MVS_Commerce.xlsx
@@ -222,25 +222,25 @@
     <t>Crear ficha administrativa global: licencia, módulos, sucursales, usuarios, consumo de límites, fechas y acciones de administración.</t>
   </si>
   <si>
+    <t>M02,M06,M07,M08</t>
+  </si>
+  <si>
+    <t>MVS administra contrato y capacidad de cada empresa desde una ficha única.</t>
+  </si>
+  <si>
+    <t>Ficha única permite cambiar licencia/límites/módulos/estado y ver propietario, uso, usuarios, fechas e historial sin entrar al tenant. Evidencia: PlatformAdminTest + CompanyLicenseTest + M02PlatformTenantListTest (17 pruebas, 98 aserciones).</t>
+  </si>
+  <si>
+    <t>M10</t>
+  </si>
+  <si>
+    <t>Auditoría y seguridad</t>
+  </si>
+  <si>
+    <t>Registrar cambios de licencia/estado/módulos/límites y reforzar aislamiento Platform/Tenant.</t>
+  </si>
+  <si>
     <t>PENDIENTE</t>
-  </si>
-  <si>
-    <t>M02,M06,M07,M08</t>
-  </si>
-  <si>
-    <t>MVS administra contrato y capacidad de cada empresa desde una ficha única.</t>
-  </si>
-  <si>
-    <t>Desde una empresa se pueden cambiar límites/módulos/estado y ver uso actual sin editar datos operativos.</t>
-  </si>
-  <si>
-    <t>M10</t>
-  </si>
-  <si>
-    <t>Auditoría y seguridad</t>
-  </si>
-  <si>
-    <t>Registrar cambios de licencia/estado/módulos/límites y reforzar aislamiento Platform/Tenant.</t>
   </si>
   <si>
     <t>M03-M09</t>
@@ -1124,33 +1124,33 @@
         <v>62</v>
       </c>
       <c r="E17" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="F17" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="F17" s="8" t="s">
+      <c r="G17" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="G17" s="8" t="s">
+      <c r="H17" s="8" t="s">
         <v>70</v>
-      </c>
-      <c r="H17" s="8" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="18" spans="1:8">
       <c r="A18" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="B18" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="B18" s="8" t="s">
+      <c r="C18" s="8" t="s">
         <v>73</v>
-      </c>
-      <c r="C18" s="8" t="s">
-        <v>74</v>
       </c>
       <c r="D18" s="8" t="s">
         <v>17</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="F18" s="8" t="s">
         <v>75</v>
@@ -1176,7 +1176,7 @@
         <v>62</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="F19" s="8" t="s">
         <v>81</v>
@@ -1202,7 +1202,7 @@
         <v>17</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="F20" s="8" t="s">
         <v>87</v>

</xml_diff>

<commit_message>
feat: completar auditoria administrativa M10
</commit_message>
<xml_diff>
--- a/docs/Cronograma_M_Panel_Maestro_MVS_Commerce.xlsx
+++ b/docs/Cronograma_M_Panel_Maestro_MVS_Commerce.xlsx
@@ -240,25 +240,25 @@
     <t>Registrar cambios de licencia/estado/módulos/límites y reforzar aislamiento Platform/Tenant.</t>
   </si>
   <si>
+    <t>M03-M09</t>
+  </si>
+  <si>
+    <t>Trazabilidad de quién cambió qué y cuándo; ningún tenant ve/edita otro tenant o privilegios de plataforma.</t>
+  </si>
+  <si>
+    <t>Auditoría con actor/empresa/snapshot para licencia, estado, límites y módulos; aislamiento y escalada sin fallos. Evidencia: M10PlatformAuditSecurityTest + M01/PlatformAdmin/módulos (24 pruebas, 122 aserciones).</t>
+  </si>
+  <si>
+    <t>M11</t>
+  </si>
+  <si>
+    <t>UX responsive</t>
+  </si>
+  <si>
+    <t>Pulir Panel Maestro y onboarding para escritorio/tablet/móvil, acciones claras y sin mezclar responsabilidades.</t>
+  </si>
+  <si>
     <t>PENDIENTE</t>
-  </si>
-  <si>
-    <t>M03-M09</t>
-  </si>
-  <si>
-    <t>Trazabilidad de quién cambió qué y cuándo; ningún tenant ve/edita otro tenant o privilegios de plataforma.</t>
-  </si>
-  <si>
-    <t>Pruebas de aislamiento, escalada de privilegios y auditoría sin fallos.</t>
-  </si>
-  <si>
-    <t>M11</t>
-  </si>
-  <si>
-    <t>UX responsive</t>
-  </si>
-  <si>
-    <t>Pulir Panel Maestro y onboarding para escritorio/tablet/móvil, acciones claras y sin mezclar responsabilidades.</t>
   </si>
   <si>
     <t>M03-M10</t>
@@ -1150,33 +1150,33 @@
         <v>17</v>
       </c>
       <c r="E18" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="F18" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="F18" s="8" t="s">
+      <c r="G18" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="G18" s="8" t="s">
+      <c r="H18" s="8" t="s">
         <v>76</v>
-      </c>
-      <c r="H18" s="8" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="19" spans="1:8">
       <c r="A19" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="B19" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="B19" s="8" t="s">
+      <c r="C19" s="8" t="s">
         <v>79</v>
-      </c>
-      <c r="C19" s="8" t="s">
-        <v>80</v>
       </c>
       <c r="D19" s="8" t="s">
         <v>62</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="F19" s="8" t="s">
         <v>81</v>
@@ -1202,7 +1202,7 @@
         <v>17</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="F20" s="8" t="s">
         <v>87</v>

</xml_diff>

<commit_message>
docs: completar experiencia responsive M11
</commit_message>
<xml_diff>
--- a/docs/Cronograma_M_Panel_Maestro_MVS_Commerce.xlsx
+++ b/docs/Cronograma_M_Panel_Maestro_MVS_Commerce.xlsx
@@ -258,25 +258,25 @@
     <t>Pulir Panel Maestro y onboarding para escritorio/tablet/móvil, acciones claras y sin mezclar responsabilidades.</t>
   </si>
   <si>
+    <t>M03-M10</t>
+  </si>
+  <si>
+    <t>Experiencia SaaS profesional y escalable.</t>
+  </si>
+  <si>
+    <t>Dashboard, alta, ficha y onboarding sin overflow, controles táctiles y grids 360/768/1280. Evidencia: UI Panel/onboarding/navegación (14 pruebas, 66 aserciones) + build Vite.</t>
+  </si>
+  <si>
+    <t>M12</t>
+  </si>
+  <si>
+    <t>Regresión y despliegue</t>
+  </si>
+  <si>
+    <t>Ejecutar regresión, actualizar documentación, commit/push, desplegar y usar MYM como primer tenant real.</t>
+  </si>
+  <si>
     <t>PENDIENTE</t>
-  </si>
-  <si>
-    <t>M03-M10</t>
-  </si>
-  <si>
-    <t>Experiencia SaaS profesional y escalable.</t>
-  </si>
-  <si>
-    <t>Sin overflow; acciones críticas claras; formularios y tablas responsivos.</t>
-  </si>
-  <si>
-    <t>M12</t>
-  </si>
-  <si>
-    <t>Regresión y despliegue</t>
-  </si>
-  <si>
-    <t>Ejecutar regresión, actualizar documentación, commit/push, desplegar y usar MYM como primer tenant real.</t>
   </si>
   <si>
     <t>M01-M11</t>
@@ -1176,33 +1176,33 @@
         <v>62</v>
       </c>
       <c r="E19" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="F19" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="F19" s="8" t="s">
+      <c r="G19" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="G19" s="8" t="s">
+      <c r="H19" s="8" t="s">
         <v>82</v>
-      </c>
-      <c r="H19" s="8" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="20" spans="1:8">
       <c r="A20" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="B20" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="B20" s="8" t="s">
+      <c r="C20" s="8" t="s">
         <v>85</v>
-      </c>
-      <c r="C20" s="8" t="s">
-        <v>86</v>
       </c>
       <c r="D20" s="8" t="s">
         <v>17</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="F20" s="8" t="s">
         <v>87</v>

</xml_diff>

<commit_message>
docs: cerrar cronograma panel maestro M12
</commit_message>
<xml_diff>
--- a/docs/Cronograma_M_Panel_Maestro_MVS_Commerce.xlsx
+++ b/docs/Cronograma_M_Panel_Maestro_MVS_Commerce.xlsx
@@ -276,7 +276,7 @@
     <t>Ejecutar regresión, actualizar documentación, commit/push, desplegar y usar MYM como primer tenant real.</t>
   </si>
   <si>
-    <t>PENDIENTE</t>
+    <t>COMPLETADO / DESPLIEGUE PENDIENTE</t>
   </si>
   <si>
     <t>M01-M11</t>
@@ -285,7 +285,7 @@
     <t>Flujo completo validado en producción antes de alta de más clientes.</t>
   </si>
   <si>
-    <t>admin@mvscommerce.com crea licencia MYM; MYM completa onboarding; 2 sucursales; módulos y suspensión funcionan.</t>
+    <t>Flujo M01–M11 validado; escenario MYM aislado cubre contrato, onboarding, 2 sucursales, módulos y suspensión. Evidencia: regresión integrada 53 pruebas, 273 aserciones; Pint, diff-check y build correctos. Producción/datos reales NO tocados; listo para aprobación.</t>
   </si>
   <si>
     <t>REGLAS NO NEGOCIABLES DEL PANEL MAESTRO</t>

</xml_diff>

<commit_message>
feat: completar licenciamiento comercial M13
</commit_message>
<xml_diff>
--- a/docs/Cronograma_M_Panel_Maestro_MVS_Commerce.xlsx
+++ b/docs/Cronograma_M_Panel_Maestro_MVS_Commerce.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="131">
   <si>
     <t>MVS COMMERCE — CRONOGRAMA M · PANEL MAESTRO / LICENCIAMIENTO SaaS</t>
   </si>
@@ -286,6 +286,42 @@
   </si>
   <si>
     <t>Flujo M01–M11 validado; escenario MYM aislado cubre contrato, onboarding, 2 sucursales, módulos y suspensión. Evidencia: regresión integrada 53 pruebas, 273 aserciones; Pint, diff-check y build correctos. Producción/datos reales NO tocados; listo para aprobación.</t>
+  </si>
+  <si>
+    <t>M13</t>
+  </si>
+  <si>
+    <t>Licenciamiento comercial y planes</t>
+  </si>
+  <si>
+    <t>Plan comercial reutilizable como plantilla; contrato efectivo por tenant con overrides independientes de sucursales, usuarios y módulos. Datos operativos del tenant en modo supervisión de solo lectura.</t>
+  </si>
+  <si>
+    <t>Migración license_plans + CompanyLicenseService::savePlan/applyPlan; pruebas focales y regresión relacionada: 43 pruebas, 245 aserciones.</t>
+  </si>
+  <si>
+    <t>2026-08-31</t>
+  </si>
+  <si>
+    <t>Local</t>
+  </si>
+  <si>
+    <t>Sin despliegue a producción.</t>
+  </si>
+  <si>
+    <t>M14</t>
+  </si>
+  <si>
+    <t>Renovaciones y ciclo de licencia</t>
+  </si>
+  <si>
+    <t>PENDIENTE</t>
+  </si>
+  <si>
+    <t>Ciclo Trial, Active, Grace, Expired, Suspended y Cancelled; renovación, gracia y trazabilidad contractual.</t>
+  </si>
+  <si>
+    <t>Pendiente de implementación y validación.</t>
   </si>
   <si>
     <t>REGLAS NO NEGOCIABLES DEL PANEL MAESTRO</t>
@@ -785,7 +821,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="true" style="0"/>
@@ -838,13 +874,13 @@
     </row>
     <row r="5" spans="1:8">
       <c r="A5" s="4">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B5" s="4">
         <v>1</v>
       </c>
       <c r="C5" s="4">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="D5" s="4">
         <v>10</v>
@@ -1212,6 +1248,54 @@
       </c>
       <c r="H20" s="8" t="s">
         <v>89</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8">
+      <c r="A21" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="B21" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="C21" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="D21" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="E21" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="F21" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="G21" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="H21" s="8" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8">
+      <c r="A22" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="D22" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="E22" s="8"/>
+      <c r="F22" s="8"/>
+      <c r="G22" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="H22" s="8" t="s">
+        <v>101</v>
       </c>
     </row>
   </sheetData>
@@ -1244,7 +1328,7 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="9" t="s">
-        <v>90</v>
+        <v>102</v>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
@@ -1252,100 +1336,100 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="5" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>92</v>
+        <v>104</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="6" t="s">
-        <v>95</v>
+        <v>107</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>96</v>
+        <v>108</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>97</v>
+        <v>109</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>98</v>
+        <v>110</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="6" t="s">
-        <v>99</v>
+        <v>111</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>100</v>
+        <v>112</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>101</v>
+        <v>113</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>102</v>
+        <v>114</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="6" t="s">
-        <v>103</v>
+        <v>115</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>104</v>
+        <v>116</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>105</v>
+        <v>117</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>106</v>
+        <v>118</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="6" t="s">
-        <v>107</v>
+        <v>119</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>108</v>
+        <v>120</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>109</v>
+        <v>121</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>110</v>
+        <v>122</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="6" t="s">
-        <v>111</v>
+        <v>123</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>112</v>
+        <v>124</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>113</v>
+        <v>125</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>114</v>
+        <v>126</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="6" t="s">
-        <v>115</v>
+        <v>127</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>116</v>
+        <v>128</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>117</v>
+        <v>129</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>118</v>
+        <v>130</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: completar ciclo de licencias M14
</commit_message>
<xml_diff>
--- a/docs/Cronograma_M_Panel_Maestro_MVS_Commerce.xlsx
+++ b/docs/Cronograma_M_Panel_Maestro_MVS_Commerce.xlsx
@@ -315,13 +315,13 @@
     <t>Renovaciones y ciclo de licencia</t>
   </si>
   <si>
-    <t>PENDIENTE</t>
-  </si>
-  <si>
     <t>Ciclo Trial, Active, Grace, Expired, Suspended y Cancelled; renovación, gracia y trazabilidad contractual.</t>
   </si>
   <si>
-    <t>Pendiente de implementación y validación.</t>
+    <t>Migración de delta contractual + CompanyLicenseService lifecycle/renew; focal: 11 pruebas/60 aserciones; regresión M relacionada: 51 pruebas/287 aserciones; Pint, Vite build y diff check verdes.</t>
+  </si>
+  <si>
+    <t>Cierre técnico local. Sin cobros ni despliegue; pausa para aprobación de producción.</t>
   </si>
   <si>
     <t>REGLAS NO NEGOCIABLES DEL PANEL MAESTRO</t>
@@ -880,7 +880,7 @@
         <v>1</v>
       </c>
       <c r="C5" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D5" s="4">
         <v>10</v>
@@ -1284,13 +1284,17 @@
         <v>98</v>
       </c>
       <c r="C22" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="D22" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="D22" s="8" t="s">
+      <c r="E22" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="E22" s="8"/>
-      <c r="F22" s="8"/>
+      <c r="F22" s="8" t="s">
+        <v>94</v>
+      </c>
       <c r="G22" s="8" t="s">
         <v>95</v>
       </c>

</xml_diff>